<commit_message>
data: W26 inventory snapshots refreshed (operator manual update)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 26/Audio_Array/Inventory Snapshot.xlsx
+++ b/data/raw/inventory/Week 26/Audio_Array/Inventory Snapshot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 26\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5E72E7-10B9-41BB-9B0F-02355CC21E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F276DCB-DD30-4CD7-BC71-6CEEEF23BE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$195</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -798,210 +798,206 @@
     <t>B0GN321RXQ</t>
   </si>
   <si>
+    <t>FBA80119</t>
+  </si>
+  <si>
+    <t>FBA80120</t>
+  </si>
+  <si>
+    <t>FBA80121</t>
+  </si>
+  <si>
+    <t>FBA80122</t>
+  </si>
+  <si>
+    <t>FBA80123</t>
+  </si>
+  <si>
+    <t>FBA80124</t>
+  </si>
+  <si>
+    <t>FBA80125</t>
+  </si>
+  <si>
+    <t>FBA80126</t>
+  </si>
+  <si>
+    <t>FBA80114</t>
+  </si>
+  <si>
+    <t>FBA80115</t>
+  </si>
+  <si>
+    <t>FBA80116</t>
+  </si>
+  <si>
+    <t>FBA80117</t>
+  </si>
+  <si>
+    <t>AMPM</t>
+  </si>
+  <si>
+    <t>FBA78986</t>
+  </si>
+  <si>
+    <t>B0CF5WXWFH</t>
+  </si>
+  <si>
+    <t>FBA76728</t>
+  </si>
+  <si>
+    <t>B0BLNCP74M</t>
+  </si>
+  <si>
+    <t>FBA76715</t>
+  </si>
+  <si>
+    <t>B0BLK31PYH</t>
+  </si>
+  <si>
+    <t>FBA79070</t>
+  </si>
+  <si>
+    <t>B0CLH7G5WH</t>
+  </si>
+  <si>
+    <t>FBA76721</t>
+  </si>
+  <si>
+    <t>B0BLKB55BM</t>
+  </si>
+  <si>
+    <t>FBA78422</t>
+  </si>
+  <si>
+    <t>B0C598MNMC</t>
+  </si>
+  <si>
+    <t>FBA76718</t>
+  </si>
+  <si>
+    <t>B0BLKD8FVG</t>
+  </si>
+  <si>
+    <t>FBA76734</t>
+  </si>
+  <si>
+    <t>B0BLKHVCDX</t>
+  </si>
+  <si>
+    <t>FBA76725</t>
+  </si>
+  <si>
+    <t>B0BLKCSJ7Z</t>
+  </si>
+  <si>
+    <t>FBA75682</t>
+  </si>
+  <si>
+    <t>B0B4FVV78V</t>
+  </si>
+  <si>
+    <t>FBA79014</t>
+  </si>
+  <si>
+    <t>B0CH4WFQF6</t>
+  </si>
+  <si>
+    <t>FBA76743</t>
+  </si>
+  <si>
+    <t>B0BLK8PXNY</t>
+  </si>
+  <si>
+    <t>FBA79013</t>
+  </si>
+  <si>
+    <t>B0CH4TDGPG</t>
+  </si>
+  <si>
+    <t>FBA78421</t>
+  </si>
+  <si>
+    <t>B0C594FZLM</t>
+  </si>
+  <si>
+    <t>FBA75685</t>
+  </si>
+  <si>
+    <t>B0B4FXDHXW</t>
+  </si>
+  <si>
+    <t>FBA76729</t>
+  </si>
+  <si>
+    <t>B0BLNDQ757</t>
+  </si>
+  <si>
+    <t>FBA76735</t>
+  </si>
+  <si>
+    <t>B0BLKGPL4X</t>
+  </si>
+  <si>
+    <t>FBA76736</t>
+  </si>
+  <si>
+    <t>B0BLS63XCL</t>
+  </si>
+  <si>
+    <t>FBA76741</t>
+  </si>
+  <si>
+    <t>B0BLS2HJ68</t>
+  </si>
+  <si>
+    <t>FBA78424</t>
+  </si>
+  <si>
+    <t>B0C55MY66L</t>
+  </si>
+  <si>
+    <t>FBA78419</t>
+  </si>
+  <si>
+    <t>B0C55M2GBN</t>
+  </si>
+  <si>
+    <t>FBA76737</t>
+  </si>
+  <si>
+    <t>B0C59G1C4N</t>
+  </si>
+  <si>
+    <t>FBA76732</t>
+  </si>
+  <si>
+    <t>B0BLKCB2JY</t>
+  </si>
+  <si>
+    <t>B2B - AMPM</t>
+  </si>
+  <si>
+    <t>Blinkit</t>
+  </si>
+  <si>
+    <t>YNT</t>
+  </si>
+  <si>
+    <t>FBA80181</t>
+  </si>
+  <si>
     <t>Pipeline</t>
   </si>
   <si>
-    <t>FBA80119</t>
-  </si>
-  <si>
-    <t>FBA80120</t>
-  </si>
-  <si>
-    <t>FBA80121</t>
-  </si>
-  <si>
-    <t>FBA80122</t>
-  </si>
-  <si>
-    <t>FBA80123</t>
-  </si>
-  <si>
-    <t>FBA80124</t>
-  </si>
-  <si>
-    <t>FBA80125</t>
-  </si>
-  <si>
-    <t>FBA80126</t>
-  </si>
-  <si>
-    <t>FBA80114</t>
-  </si>
-  <si>
-    <t>FBA80115</t>
-  </si>
-  <si>
-    <t>FBA80116</t>
-  </si>
-  <si>
-    <t>FBA80117</t>
-  </si>
-  <si>
     <t>Open Order</t>
-  </si>
-  <si>
-    <t>AMPM</t>
-  </si>
-  <si>
-    <t>FBA78986</t>
-  </si>
-  <si>
-    <t>B0CF5WXWFH</t>
-  </si>
-  <si>
-    <t>FBA76728</t>
-  </si>
-  <si>
-    <t>B0BLNCP74M</t>
-  </si>
-  <si>
-    <t>FBA76715</t>
-  </si>
-  <si>
-    <t>B0BLK31PYH</t>
-  </si>
-  <si>
-    <t>FBA79070</t>
-  </si>
-  <si>
-    <t>B0CLH7G5WH</t>
-  </si>
-  <si>
-    <t>FBA76721</t>
-  </si>
-  <si>
-    <t>B0BLKB55BM</t>
-  </si>
-  <si>
-    <t>FBA78422</t>
-  </si>
-  <si>
-    <t>B0C598MNMC</t>
-  </si>
-  <si>
-    <t>FBA76718</t>
-  </si>
-  <si>
-    <t>B0BLKD8FVG</t>
-  </si>
-  <si>
-    <t>FBA76734</t>
-  </si>
-  <si>
-    <t>B0BLKHVCDX</t>
-  </si>
-  <si>
-    <t>FBA76725</t>
-  </si>
-  <si>
-    <t>B0BLKCSJ7Z</t>
-  </si>
-  <si>
-    <t>FBA75682</t>
-  </si>
-  <si>
-    <t>B0B4FVV78V</t>
-  </si>
-  <si>
-    <t>FBA79014</t>
-  </si>
-  <si>
-    <t>B0CH4WFQF6</t>
-  </si>
-  <si>
-    <t>FBA76743</t>
-  </si>
-  <si>
-    <t>B0BLK8PXNY</t>
-  </si>
-  <si>
-    <t>FBA79013</t>
-  </si>
-  <si>
-    <t>B0CH4TDGPG</t>
-  </si>
-  <si>
-    <t>FBA78421</t>
-  </si>
-  <si>
-    <t>B0C594FZLM</t>
-  </si>
-  <si>
-    <t>FBA75685</t>
-  </si>
-  <si>
-    <t>B0B4FXDHXW</t>
-  </si>
-  <si>
-    <t>FBA76729</t>
-  </si>
-  <si>
-    <t>B0BLNDQ757</t>
-  </si>
-  <si>
-    <t>FBA76735</t>
-  </si>
-  <si>
-    <t>B0BLKGPL4X</t>
-  </si>
-  <si>
-    <t>FBA76736</t>
-  </si>
-  <si>
-    <t>B0BLS63XCL</t>
-  </si>
-  <si>
-    <t>FBA76741</t>
-  </si>
-  <si>
-    <t>B0BLS2HJ68</t>
-  </si>
-  <si>
-    <t>FBA78424</t>
-  </si>
-  <si>
-    <t>B0C55MY66L</t>
-  </si>
-  <si>
-    <t>FBA78419</t>
-  </si>
-  <si>
-    <t>B0C55M2GBN</t>
-  </si>
-  <si>
-    <t>FBA76737</t>
-  </si>
-  <si>
-    <t>B0C59G1C4N</t>
-  </si>
-  <si>
-    <t>FBA76732</t>
-  </si>
-  <si>
-    <t>B0BLKCB2JY</t>
-  </si>
-  <si>
-    <t>B2B - AMPM</t>
-  </si>
-  <si>
-    <t>Blinkit</t>
-  </si>
-  <si>
-    <t>YNT</t>
-  </si>
-  <si>
-    <t>FBA80181</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1054,12 +1050,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF1F2937"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF1F2937"/>
       <name val="Calibri"/>
@@ -1092,7 +1082,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1115,40 +1105,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1171,57 +1134,25 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Comma" xfId="3" builtinId="3"/>
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{697FC575-8A7C-4715-A8F0-2950C62D8576}"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1782,7 +1713,7 @@
         <v>1472</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1799,7 +1730,7 @@
         <v>518</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1816,7 +1747,7 @@
         <v>1767</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1833,7 +1764,7 @@
         <v>1891</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1850,7 +1781,7 @@
         <v>259</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1867,7 +1798,7 @@
         <v>534</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1884,7 +1815,7 @@
         <v>238</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1901,7 +1832,7 @@
         <v>26</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1918,7 +1849,7 @@
         <v>44</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1935,7 +1866,7 @@
         <v>41</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1952,7 +1883,7 @@
         <v>174</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1969,7 +1900,7 @@
         <v>1219</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1986,7 +1917,7 @@
         <v>2495</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2003,7 +1934,7 @@
         <v>67</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2020,7 +1951,7 @@
         <v>355</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2037,7 +1968,7 @@
         <v>267</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2054,7 +1985,7 @@
         <v>253</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2071,7 +2002,7 @@
         <v>111</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2088,7 +2019,7 @@
         <v>2084</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2105,7 +2036,7 @@
         <v>347</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2122,7 +2053,7 @@
         <v>151</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2139,7 +2070,7 @@
         <v>136</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2156,7 +2087,7 @@
         <v>545</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2173,7 +2104,7 @@
         <v>20</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2190,7 +2121,7 @@
         <v>6</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2207,7 +2138,7 @@
         <v>104</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2224,7 +2155,7 @@
         <v>111</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2241,7 +2172,7 @@
         <v>504</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2258,7 +2189,7 @@
         <v>67</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2275,7 +2206,7 @@
         <v>76</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2292,7 +2223,7 @@
         <v>467</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2309,7 +2240,7 @@
         <v>338</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2326,7 +2257,7 @@
         <v>690</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2343,7 +2274,7 @@
         <v>803</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2360,7 +2291,7 @@
         <v>683</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2377,7 +2308,7 @@
         <v>4</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2394,7 +2325,7 @@
         <v>18</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2411,7 +2342,7 @@
         <v>23</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2428,7 +2359,7 @@
         <v>7</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2445,7 +2376,7 @@
         <v>33</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2462,7 +2393,7 @@
         <v>390</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2479,7 +2410,7 @@
         <v>288</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2496,7 +2427,7 @@
         <v>18</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2513,7 +2444,7 @@
         <v>262</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2530,7 +2461,7 @@
         <v>822</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2547,7 +2478,7 @@
         <v>1495</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2564,7 +2495,7 @@
         <v>59</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2581,7 +2512,7 @@
         <v>1</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2598,15 +2529,15 @@
         <v>7</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>234</v>
@@ -2615,15 +2546,15 @@
         <v>7</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>234</v>
@@ -2632,7 +2563,7 @@
         <v>2</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2649,7 +2580,7 @@
         <v>59</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2666,7 +2597,7 @@
         <v>233</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2683,7 +2614,7 @@
         <v>6</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2700,7 +2631,7 @@
         <v>89</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2717,7 +2648,7 @@
         <v>7</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2734,15 +2665,15 @@
         <v>8</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>234</v>
@@ -2751,7 +2682,7 @@
         <v>3</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2768,15 +2699,15 @@
         <v>8</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>234</v>
@@ -2785,15 +2716,15 @@
         <v>6</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>234</v>
@@ -2802,7 +2733,7 @@
         <v>1</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2819,15 +2750,15 @@
         <v>6</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>234</v>
@@ -2836,15 +2767,15 @@
         <v>5</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>234</v>
@@ -2853,15 +2784,15 @@
         <v>4</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>234</v>
@@ -2870,7 +2801,7 @@
         <v>3</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2887,15 +2818,15 @@
         <v>7</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C68" s="5" t="s">
         <v>234</v>
@@ -2904,15 +2835,15 @@
         <v>3</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C69" s="5" t="s">
         <v>234</v>
@@ -2921,15 +2852,15 @@
         <v>1</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>234</v>
@@ -2938,7 +2869,7 @@
         <v>3</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2955,15 +2886,15 @@
         <v>15</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>234</v>
@@ -2972,15 +2903,15 @@
         <v>3</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C73" s="5" t="s">
         <v>234</v>
@@ -2989,15 +2920,15 @@
         <v>1</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C74" s="5" t="s">
         <v>234</v>
@@ -3006,15 +2937,15 @@
         <v>2</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C75" s="5" t="s">
         <v>234</v>
@@ -3023,7 +2954,7 @@
         <v>1</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3040,15 +2971,15 @@
         <v>1783</v>
       </c>
       <c r="J76" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C77" s="5" t="s">
         <v>234</v>
@@ -3057,15 +2988,15 @@
         <v>1</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="78" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>234</v>
@@ -3074,15 +3005,15 @@
         <v>1</v>
       </c>
       <c r="J78" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>234</v>
@@ -3091,15 +3022,15 @@
         <v>3</v>
       </c>
       <c r="J79" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C80" s="5" t="s">
         <v>234</v>
@@ -3108,7 +3039,7 @@
         <v>1</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3125,15 +3056,15 @@
         <v>147</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>234</v>
@@ -3142,15 +3073,15 @@
         <v>2</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="83" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C83" s="5" t="s">
         <v>234</v>
@@ -3159,15 +3090,15 @@
         <v>4</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="84" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C84" s="5" t="s">
         <v>234</v>
@@ -3176,15 +3107,15 @@
         <v>3</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="85" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C85" s="5" t="s">
         <v>234</v>
@@ -3193,7 +3124,7 @@
         <v>1</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3210,7 +3141,7 @@
         <v>182</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="87" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3227,7 +3158,7 @@
         <v>1473</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="88" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3244,7 +3175,7 @@
         <v>495</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="89" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3261,7 +3192,7 @@
         <v>1730</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="90" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3278,7 +3209,7 @@
         <v>738</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3295,7 +3226,7 @@
         <v>174</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3312,7 +3243,7 @@
         <v>921</v>
       </c>
       <c r="J92" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="93" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3329,7 +3260,7 @@
         <v>1516</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="94" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3346,7 +3277,7 @@
         <v>1342</v>
       </c>
       <c r="J94" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3363,7 +3294,7 @@
         <v>416</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3380,7 +3311,7 @@
         <v>516</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3397,7 +3328,7 @@
         <v>1154</v>
       </c>
       <c r="J97" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3414,7 +3345,7 @@
         <v>255</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3431,7 +3362,7 @@
         <v>250</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3448,7 +3379,7 @@
         <v>5</v>
       </c>
       <c r="J100" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3465,7 +3396,7 @@
         <v>3</v>
       </c>
       <c r="J101" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="102" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3482,7 +3413,7 @@
         <v>16</v>
       </c>
       <c r="J102" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="103" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3499,7 +3430,7 @@
         <v>337</v>
       </c>
       <c r="J103" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="104" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3516,7 +3447,7 @@
         <v>324</v>
       </c>
       <c r="J104" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="105" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3533,7 +3464,7 @@
         <v>224</v>
       </c>
       <c r="J105" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="106" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3550,7 +3481,7 @@
         <v>593</v>
       </c>
       <c r="J106" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="107" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3567,7 +3498,7 @@
         <v>798</v>
       </c>
       <c r="J107" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="108" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3584,7 +3515,7 @@
         <v>217</v>
       </c>
       <c r="J108" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="109" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3601,7 +3532,7 @@
         <v>52</v>
       </c>
       <c r="J109" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="110" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3618,7 +3549,7 @@
         <v>1</v>
       </c>
       <c r="J110" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="111" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3635,7 +3566,7 @@
         <v>9</v>
       </c>
       <c r="J111" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3652,7 +3583,7 @@
         <v>396</v>
       </c>
       <c r="J112" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3669,7 +3600,7 @@
         <v>420</v>
       </c>
       <c r="J113" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="114" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3686,7 +3617,7 @@
         <v>185</v>
       </c>
       <c r="J114" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3703,7 +3634,7 @@
         <v>185</v>
       </c>
       <c r="J115" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="116" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3720,7 +3651,7 @@
         <v>23</v>
       </c>
       <c r="J116" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="117" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3737,7 +3668,7 @@
         <v>11</v>
       </c>
       <c r="J117" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3754,7 +3685,7 @@
         <v>7</v>
       </c>
       <c r="J118" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3771,7 +3702,7 @@
         <v>124</v>
       </c>
       <c r="J119" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3788,7 +3719,7 @@
         <v>165</v>
       </c>
       <c r="J120" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3805,7 +3736,7 @@
         <v>65</v>
       </c>
       <c r="J121" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3822,7 +3753,7 @@
         <v>64</v>
       </c>
       <c r="J122" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3839,7 +3770,7 @@
         <v>15</v>
       </c>
       <c r="J123" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3856,7 +3787,7 @@
         <v>15</v>
       </c>
       <c r="J124" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3873,840 +3804,840 @@
         <v>286</v>
       </c>
       <c r="J125" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="13" t="s">
+      <c r="A126" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B126" s="14" t="s">
+      <c r="B126" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="C126" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I126" s="13">
+      <c r="C126" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I126" s="8">
         <v>6</v>
       </c>
       <c r="J126" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="13" t="s">
+      <c r="A127" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B127" s="14" t="s">
+      <c r="B127" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="C127" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I127" s="13">
+      <c r="C127" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I127" s="8">
         <v>1</v>
       </c>
       <c r="J127" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="128" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="13" t="s">
+      <c r="A128" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B128" s="14" t="s">
+      <c r="B128" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C128" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I128" s="13">
+      <c r="C128" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I128" s="8">
         <v>33</v>
       </c>
       <c r="J128" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="13" t="s">
+      <c r="A129" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B129" s="14" t="s">
+      <c r="B129" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="C129" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I129" s="13">
+      <c r="C129" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I129" s="8">
         <v>5</v>
       </c>
       <c r="J129" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="130" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="13" t="s">
+      <c r="A130" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B130" s="14" t="s">
+      <c r="B130" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C130" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I130" s="13">
+      <c r="C130" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I130" s="8">
         <v>7</v>
       </c>
       <c r="J130" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="131" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="13" t="s">
+      <c r="A131" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B131" s="14" t="s">
+      <c r="B131" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C131" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I131" s="13">
+      <c r="C131" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I131" s="8">
         <v>2</v>
       </c>
       <c r="J131" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="132" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="13" t="s">
+      <c r="A132" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B132" s="14" t="s">
+      <c r="B132" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="C132" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I132" s="13">
+      <c r="C132" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I132" s="8">
         <v>3</v>
       </c>
       <c r="J132" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="13" t="s">
+      <c r="A133" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B133" s="14" t="s">
+      <c r="B133" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="C133" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I133" s="13">
+      <c r="C133" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I133" s="8">
         <v>3</v>
       </c>
       <c r="J133" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="13" t="s">
+      <c r="A134" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B134" s="14" t="s">
+      <c r="B134" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="C134" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I134" s="13">
+      <c r="C134" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I134" s="8">
         <v>5</v>
       </c>
       <c r="J134" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="135" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="13" t="s">
+      <c r="A135" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B135" s="14" t="s">
+      <c r="B135" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C135" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I135" s="13">
+      <c r="C135" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I135" s="8">
         <v>97</v>
       </c>
       <c r="J135" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="136" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="13" t="s">
+      <c r="A136" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B136" s="14" t="s">
+      <c r="B136" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C136" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I136" s="13">
+      <c r="C136" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I136" s="8">
         <v>3</v>
       </c>
       <c r="J136" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="13" t="s">
+      <c r="A137" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B137" s="14" t="s">
+      <c r="B137" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="C137" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I137" s="13">
+      <c r="C137" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I137" s="8">
         <v>1</v>
       </c>
       <c r="J137" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="13" t="s">
+      <c r="A138" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B138" s="14" t="s">
+      <c r="B138" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C138" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I138" s="13">
+      <c r="C138" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I138" s="8">
         <v>63</v>
       </c>
       <c r="J138" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="139" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="13" t="s">
+      <c r="A139" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B139" s="14" t="s">
+      <c r="B139" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C139" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I139" s="13">
+      <c r="C139" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I139" s="8">
         <v>108</v>
       </c>
       <c r="J139" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="140" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="13" t="s">
+      <c r="A140" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B140" s="14" t="s">
+      <c r="B140" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="C140" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I140" s="13">
+      <c r="C140" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I140" s="8">
         <v>18</v>
       </c>
       <c r="J140" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="141" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="13" t="s">
+      <c r="A141" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B141" s="14" t="s">
+      <c r="B141" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="C141" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I141" s="13">
+      <c r="C141" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I141" s="8">
         <v>24</v>
       </c>
       <c r="J141" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="13" t="s">
+      <c r="A142" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B142" s="14" t="s">
+      <c r="B142" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="C142" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I142" s="13">
+      <c r="C142" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I142" s="8">
         <v>30</v>
       </c>
       <c r="J142" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="143" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="13" t="s">
+      <c r="A143" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B143" s="14" t="s">
+      <c r="B143" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="C143" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I143" s="13">
+      <c r="C143" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I143" s="8">
         <v>42</v>
       </c>
       <c r="J143" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="13" t="s">
+      <c r="A144" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B144" s="14" t="s">
+      <c r="B144" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="C144" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I144" s="13">
+      <c r="C144" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I144" s="8">
         <v>74</v>
       </c>
       <c r="J144" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="13" t="s">
+      <c r="A145" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B145" s="14" t="s">
+      <c r="B145" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C145" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I145" s="13">
+      <c r="C145" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I145" s="8">
         <v>19</v>
       </c>
       <c r="J145" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="13" t="s">
+      <c r="A146" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B146" s="14" t="s">
+      <c r="B146" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C146" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I146" s="13">
+      <c r="C146" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I146" s="8">
         <v>16</v>
       </c>
       <c r="J146" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="13" t="s">
+      <c r="A147" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B147" s="14" t="s">
+      <c r="B147" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="C147" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I147" s="13">
+      <c r="C147" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I147" s="8">
         <v>51</v>
       </c>
       <c r="J147" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="13" t="s">
+      <c r="A148" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B148" s="14" t="s">
+      <c r="B148" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C148" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I148" s="13">
+      <c r="C148" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I148" s="8">
         <v>4</v>
       </c>
       <c r="J148" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="13" t="s">
+      <c r="A149" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B149" s="14" t="s">
+      <c r="B149" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C149" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I149" s="13">
+      <c r="C149" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I149" s="8">
         <v>3</v>
       </c>
       <c r="J149" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="150" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="13" t="s">
+      <c r="A150" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B150" s="14" t="s">
+      <c r="B150" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C150" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I150" s="13">
+      <c r="C150" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I150" s="8">
         <v>6</v>
       </c>
       <c r="J150" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="151" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="13" t="s">
+      <c r="A151" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B151" s="14" t="s">
+      <c r="B151" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="C151" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I151" s="13">
+      <c r="C151" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I151" s="8">
         <v>97</v>
       </c>
       <c r="J151" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="13" t="s">
+      <c r="A152" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B152" s="14" t="s">
+      <c r="B152" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="C152" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I152" s="13">
+      <c r="C152" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I152" s="8">
         <v>2</v>
       </c>
       <c r="J152" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="13" t="s">
+      <c r="A153" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B153" s="14" t="s">
+      <c r="B153" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C153" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I153" s="13">
+      <c r="C153" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I153" s="8">
         <v>20</v>
       </c>
       <c r="J153" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="13" t="s">
+      <c r="A154" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B154" s="14" t="s">
+      <c r="B154" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C154" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I154" s="13">
+      <c r="C154" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I154" s="8">
         <v>45</v>
       </c>
       <c r="J154" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="155" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="13" t="s">
+      <c r="A155" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B155" s="14" t="s">
+      <c r="B155" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C155" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I155" s="13">
+      <c r="C155" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I155" s="8">
         <v>3</v>
       </c>
       <c r="J155" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="156" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="13" t="s">
+      <c r="A156" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B156" s="14" t="s">
+      <c r="B156" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="C156" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I156" s="13">
+      <c r="C156" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I156" s="8">
         <v>38</v>
       </c>
       <c r="J156" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="157" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="13" t="s">
+      <c r="A157" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B157" s="14" t="s">
+      <c r="B157" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="C157" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I157" s="13">
+      <c r="C157" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I157" s="8">
         <v>5</v>
       </c>
       <c r="J157" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="13" t="s">
+      <c r="A158" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B158" s="14" t="s">
+      <c r="B158" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="C158" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I158" s="13">
+      <c r="C158" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I158" s="8">
         <v>2</v>
       </c>
       <c r="J158" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="159" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="13" t="s">
+      <c r="A159" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B159" s="14" t="s">
+      <c r="B159" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="C159" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I159" s="13">
+      <c r="C159" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I159" s="8">
         <v>9</v>
       </c>
       <c r="J159" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="160" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="13" t="s">
+      <c r="A160" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B160" s="14" t="s">
+      <c r="B160" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="C160" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I160" s="13">
+      <c r="C160" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I160" s="8">
         <v>11</v>
       </c>
       <c r="J160" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="161" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="13" t="s">
+      <c r="A161" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B161" s="14" t="s">
+      <c r="B161" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="C161" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I161" s="13">
+      <c r="C161" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I161" s="8">
         <v>9</v>
       </c>
       <c r="J161" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="162" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="13" t="s">
+      <c r="A162" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B162" s="14" t="s">
+      <c r="B162" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="C162" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I162" s="13">
+      <c r="C162" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I162" s="8">
         <v>1</v>
       </c>
       <c r="J162" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="13" t="s">
+      <c r="A163" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="B163" s="14" t="s">
+      <c r="B163" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="C163" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I163" s="13">
+      <c r="C163" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I163" s="8">
         <v>26</v>
       </c>
       <c r="J163" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="13" t="s">
+      <c r="A164" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B164" s="14" t="s">
+      <c r="B164" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="C164" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I164" s="13">
+      <c r="C164" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I164" s="8">
         <v>50</v>
       </c>
       <c r="J164" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="165" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="13" t="s">
+      <c r="A165" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B165" s="14" t="s">
+      <c r="B165" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C165" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I165" s="13">
+      <c r="C165" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I165" s="8">
         <v>2</v>
       </c>
       <c r="J165" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="166" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="13" t="s">
+      <c r="A166" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B166" s="14" t="s">
+      <c r="B166" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="C166" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I166" s="13">
+      <c r="C166" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I166" s="8">
         <v>2</v>
       </c>
       <c r="J166" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="167" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="13" t="s">
+      <c r="A167" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B167" s="14" t="s">
+      <c r="B167" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C167" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I167" s="13">
+      <c r="C167" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I167" s="8">
         <v>9</v>
       </c>
       <c r="J167" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="168" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="14" t="s">
+      <c r="A168" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B168" s="14" t="s">
+      <c r="B168" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="C168" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I168" s="13">
+      <c r="C168" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I168" s="8">
         <v>4</v>
       </c>
       <c r="J168" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="169" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="14" t="s">
+      <c r="A169" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B169" s="14" t="s">
+      <c r="B169" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="C169" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I169" s="13">
+      <c r="C169" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I169" s="8">
         <v>5</v>
       </c>
       <c r="J169" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="170" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="14" t="s">
+      <c r="A170" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="B170" s="14" t="s">
+      <c r="B170" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="C170" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I170" s="13">
+      <c r="C170" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I170" s="8">
         <v>3</v>
       </c>
       <c r="J170" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="171" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A171" s="14" t="s">
+      <c r="A171" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B171" s="14" t="s">
+      <c r="B171" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="C171" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I171" s="13">
+      <c r="C171" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I171" s="8">
         <v>5</v>
       </c>
       <c r="J171" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="172" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A172" s="14" t="s">
+      <c r="A172" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B172" s="14" t="s">
+      <c r="B172" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="C172" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I172" s="13">
+      <c r="C172" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I172" s="8">
         <v>49</v>
       </c>
       <c r="J172" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="173" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="13" t="s">
+      <c r="A173" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B173" s="14" t="s">
+      <c r="B173" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="C173" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I173" s="13">
+      <c r="C173" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I173" s="8">
         <v>3</v>
       </c>
       <c r="J173" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="174" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="13" t="s">
+      <c r="A174" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B174" s="14" t="s">
+      <c r="B174" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="C174" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="I174" s="13">
+      <c r="C174" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="I174" s="8">
         <v>3</v>
       </c>
       <c r="J174" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="175" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -4723,9 +4654,9 @@
         <v>69</v>
       </c>
       <c r="J175" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K175" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K175" s="10"/>
     </row>
     <row r="176" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="3" t="s">
@@ -4741,9 +4672,9 @@
         <v>183</v>
       </c>
       <c r="J176" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K176" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K176" s="10"/>
     </row>
     <row r="177" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="3" t="s">
@@ -4759,9 +4690,9 @@
         <v>28</v>
       </c>
       <c r="J177" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K177" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K177" s="10"/>
     </row>
     <row r="178" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="3" t="s">
@@ -4777,9 +4708,9 @@
         <v>49</v>
       </c>
       <c r="J178" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K178" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K178" s="10"/>
     </row>
     <row r="179" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="3" t="s">
@@ -4795,9 +4726,9 @@
         <v>25</v>
       </c>
       <c r="J179" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K179" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K179" s="10"/>
     </row>
     <row r="180" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="3" t="s">
@@ -4813,9 +4744,9 @@
         <v>24</v>
       </c>
       <c r="J180" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K180" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K180" s="10"/>
     </row>
     <row r="181" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="3" t="s">
@@ -4831,9 +4762,9 @@
         <v>7</v>
       </c>
       <c r="J181" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="K181" s="15"/>
+        <v>313</v>
+      </c>
+      <c r="K181" s="10"/>
     </row>
     <row r="182" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="3" t="s">
@@ -4849,9 +4780,9 @@
         <v>2</v>
       </c>
       <c r="J182" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K182" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K182" s="10"/>
     </row>
     <row r="183" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="3" t="s">
@@ -4867,9 +4798,9 @@
         <v>24</v>
       </c>
       <c r="J183" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K183" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K183" s="10"/>
     </row>
     <row r="184" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="3" t="s">
@@ -4885,9 +4816,9 @@
         <v>4</v>
       </c>
       <c r="J184" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K184" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K184" s="10"/>
     </row>
     <row r="185" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="3" t="s">
@@ -4903,9 +4834,9 @@
         <v>10</v>
       </c>
       <c r="J185" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K185" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K185" s="10"/>
     </row>
     <row r="186" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="3" t="s">
@@ -4921,9 +4852,9 @@
         <v>5</v>
       </c>
       <c r="J186" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K186" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K186" s="10"/>
     </row>
     <row r="187" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="3" t="s">
@@ -4939,9 +4870,9 @@
         <v>9</v>
       </c>
       <c r="J187" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K187" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K187" s="10"/>
     </row>
     <row r="188" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="3" t="s">
@@ -4957,9 +4888,9 @@
         <v>10</v>
       </c>
       <c r="J188" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K188" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K188" s="10"/>
     </row>
     <row r="189" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="3" t="s">
@@ -4975,9 +4906,9 @@
         <v>4</v>
       </c>
       <c r="J189" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K189" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K189" s="10"/>
     </row>
     <row r="190" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="3" t="s">
@@ -4993,9 +4924,9 @@
         <v>30</v>
       </c>
       <c r="J190" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K190" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K190" s="10"/>
     </row>
     <row r="191" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="3" t="s">
@@ -5011,9 +4942,9 @@
         <v>3</v>
       </c>
       <c r="J191" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K191" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K191" s="10"/>
     </row>
     <row r="192" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="3" t="s">
@@ -5029,9 +4960,9 @@
         <v>3</v>
       </c>
       <c r="J192" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K192" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K192" s="10"/>
     </row>
     <row r="193" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="3" t="s">
@@ -5047,12 +4978,12 @@
         <v>3</v>
       </c>
       <c r="J193" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K193" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K193" s="10"/>
     </row>
     <row r="194" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A194" s="16" t="s">
+      <c r="A194" s="11" t="s">
         <v>82</v>
       </c>
       <c r="B194" s="3" t="s">
@@ -5065,9 +4996,9 @@
         <v>25</v>
       </c>
       <c r="J194" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="K194" s="15"/>
+        <v>314</v>
+      </c>
+      <c r="K194" s="10"/>
     </row>
     <row r="195" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="3" t="s">
@@ -5083,840 +5014,775 @@
         <v>5</v>
       </c>
       <c r="J195" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="K195" s="10"/>
+    </row>
+    <row r="196" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>76</v>
+      </c>
+      <c r="B196" t="s">
+        <v>187</v>
+      </c>
+      <c r="C196" t="s">
+        <v>234</v>
+      </c>
+      <c r="I196">
+        <v>1496</v>
+      </c>
+      <c r="J196" t="s">
         <v>316</v>
       </c>
-      <c r="K195" s="15"/>
-    </row>
-    <row r="196" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A196" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B196" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C196" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I196" s="9">
-        <v>1496</v>
-      </c>
-      <c r="J196" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K196" s="8"/>
-    </row>
-    <row r="197" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A197" s="4" t="s">
+    </row>
+    <row r="197" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
         <v>50</v>
       </c>
-      <c r="B197" s="4" t="s">
+      <c r="B197" t="s">
         <v>161</v>
       </c>
-      <c r="C197" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I197" s="9">
+      <c r="C197" t="s">
+        <v>234</v>
+      </c>
+      <c r="I197">
         <v>1000</v>
       </c>
-      <c r="J197" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K197" s="8"/>
-    </row>
-    <row r="198" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="4" t="s">
+      <c r="J197" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="198" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
         <v>59</v>
       </c>
-      <c r="B198" s="4" t="s">
+      <c r="B198" t="s">
         <v>170</v>
       </c>
-      <c r="C198" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I198" s="9">
+      <c r="C198" t="s">
+        <v>234</v>
+      </c>
+      <c r="I198">
         <v>1000</v>
       </c>
-      <c r="J198" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K198" s="8"/>
-    </row>
-    <row r="199" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A199" s="4" t="s">
+      <c r="J198" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="199" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
         <v>46</v>
       </c>
-      <c r="B199" s="4" t="s">
+      <c r="B199" t="s">
         <v>157</v>
       </c>
-      <c r="C199" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I199" s="9">
+      <c r="C199" t="s">
+        <v>234</v>
+      </c>
+      <c r="I199">
         <v>504</v>
       </c>
-      <c r="J199" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K199" s="8"/>
-    </row>
-    <row r="200" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="6" t="s">
+      <c r="J199" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="200" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
         <v>97</v>
       </c>
-      <c r="B200" s="3" t="s">
+      <c r="B200" t="s">
         <v>208</v>
       </c>
-      <c r="C200" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I200" s="9">
+      <c r="C200" t="s">
+        <v>234</v>
+      </c>
+      <c r="I200">
         <v>1300</v>
       </c>
-      <c r="J200" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K200" s="8"/>
-    </row>
-    <row r="201" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="6" t="s">
+      <c r="J200" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="201" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
         <v>241</v>
       </c>
-      <c r="B201" s="11" t="s">
+      <c r="B201" t="s">
         <v>242</v>
       </c>
-      <c r="C201" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I201" s="12">
+      <c r="C201" t="s">
+        <v>234</v>
+      </c>
+      <c r="I201">
         <v>200</v>
       </c>
-      <c r="J201" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K201" s="8"/>
-    </row>
-    <row r="202" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="6" t="s">
+      <c r="J201" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="202" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
         <v>99</v>
       </c>
-      <c r="B202" s="11" t="s">
+      <c r="B202" t="s">
         <v>210</v>
       </c>
-      <c r="C202" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I202" s="12">
+      <c r="C202" t="s">
+        <v>234</v>
+      </c>
+      <c r="I202">
         <v>40</v>
       </c>
-      <c r="J202" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K202" s="8"/>
-    </row>
-    <row r="203" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A203" s="6" t="s">
+      <c r="J202" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="203" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
         <v>100</v>
       </c>
-      <c r="B203" s="11" t="s">
+      <c r="B203" t="s">
         <v>211</v>
       </c>
-      <c r="C203" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I203" s="12">
+      <c r="C203" t="s">
+        <v>234</v>
+      </c>
+      <c r="I203">
         <v>50</v>
       </c>
-      <c r="J203" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K203" s="8"/>
-    </row>
-    <row r="204" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A204" s="6" t="s">
+      <c r="J203" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="204" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
         <v>101</v>
       </c>
-      <c r="B204" s="11" t="s">
+      <c r="B204" t="s">
         <v>212</v>
       </c>
-      <c r="C204" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I204" s="12">
+      <c r="C204" t="s">
+        <v>234</v>
+      </c>
+      <c r="I204">
         <v>300</v>
       </c>
-      <c r="J204" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K204" s="8"/>
-    </row>
-    <row r="205" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A205" s="6" t="s">
+      <c r="J204" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="205" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
         <v>102</v>
       </c>
-      <c r="B205" s="3" t="s">
+      <c r="B205" t="s">
         <v>213</v>
       </c>
-      <c r="C205" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I205" s="9">
+      <c r="C205" t="s">
+        <v>234</v>
+      </c>
+      <c r="I205">
         <v>200</v>
       </c>
-      <c r="J205" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K205" s="8"/>
-    </row>
-    <row r="206" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A206" s="6" t="s">
+      <c r="J205" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="206" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
         <v>122</v>
       </c>
-      <c r="B206" s="3" t="s">
+      <c r="B206" t="s">
         <v>233</v>
       </c>
-      <c r="C206" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I206" s="9">
+      <c r="C206" t="s">
+        <v>234</v>
+      </c>
+      <c r="I206">
         <v>300</v>
       </c>
-      <c r="J206" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="K206" s="8"/>
-    </row>
-    <row r="207" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A207" s="4" t="s">
+      <c r="J206" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="207" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
         <v>12</v>
       </c>
-      <c r="B207" s="4" t="s">
+      <c r="B207" t="s">
         <v>123</v>
       </c>
-      <c r="C207" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I207" s="9">
+      <c r="C207" t="s">
+        <v>234</v>
+      </c>
+      <c r="I207">
         <v>5004</v>
       </c>
-      <c r="J207" s="7" t="s">
+      <c r="J207" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="208" spans="1:11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>20</v>
+      </c>
+      <c r="B208" t="s">
+        <v>131</v>
+      </c>
+      <c r="C208" t="s">
+        <v>234</v>
+      </c>
+      <c r="I208">
+        <v>500</v>
+      </c>
+      <c r="J208" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="209" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>70</v>
+      </c>
+      <c r="B209" t="s">
+        <v>181</v>
+      </c>
+      <c r="C209" t="s">
+        <v>234</v>
+      </c>
+      <c r="I209">
+        <v>1000</v>
+      </c>
+      <c r="J209" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="210" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>61</v>
+      </c>
+      <c r="B210" t="s">
+        <v>172</v>
+      </c>
+      <c r="C210" t="s">
+        <v>234</v>
+      </c>
+      <c r="I210">
+        <v>1000</v>
+      </c>
+      <c r="J210" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="211" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>36</v>
+      </c>
+      <c r="B211" t="s">
+        <v>147</v>
+      </c>
+      <c r="C211" t="s">
+        <v>234</v>
+      </c>
+      <c r="I211">
+        <v>2010</v>
+      </c>
+      <c r="J211" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="212" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>30</v>
+      </c>
+      <c r="B212" t="s">
+        <v>141</v>
+      </c>
+      <c r="C212" t="s">
+        <v>234</v>
+      </c>
+      <c r="I212">
+        <v>504</v>
+      </c>
+      <c r="J212" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="213" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>48</v>
+      </c>
+      <c r="B213" t="s">
+        <v>159</v>
+      </c>
+      <c r="C213" t="s">
+        <v>234</v>
+      </c>
+      <c r="I213">
+        <v>501</v>
+      </c>
+      <c r="J213" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="214" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>54</v>
+      </c>
+      <c r="B214" t="s">
+        <v>165</v>
+      </c>
+      <c r="C214" t="s">
+        <v>234</v>
+      </c>
+      <c r="I214">
+        <v>504</v>
+      </c>
+      <c r="J214" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="215" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>50</v>
+      </c>
+      <c r="B215" t="s">
+        <v>161</v>
+      </c>
+      <c r="C215" t="s">
+        <v>234</v>
+      </c>
+      <c r="I215">
+        <v>1000</v>
+      </c>
+      <c r="J215" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="216" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>22</v>
+      </c>
+      <c r="B216" t="s">
+        <v>133</v>
+      </c>
+      <c r="C216" t="s">
+        <v>234</v>
+      </c>
+      <c r="I216">
+        <v>480</v>
+      </c>
+      <c r="J216" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="217" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>13</v>
+      </c>
+      <c r="B217" t="s">
+        <v>124</v>
+      </c>
+      <c r="C217" t="s">
+        <v>234</v>
+      </c>
+      <c r="I217">
+        <v>504</v>
+      </c>
+      <c r="J217" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="218" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>23</v>
+      </c>
+      <c r="B218" t="s">
+        <v>134</v>
+      </c>
+      <c r="C218" t="s">
+        <v>234</v>
+      </c>
+      <c r="I218">
+        <v>500</v>
+      </c>
+      <c r="J218" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="219" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>34</v>
+      </c>
+      <c r="B219" t="s">
+        <v>145</v>
+      </c>
+      <c r="C219" t="s">
+        <v>234</v>
+      </c>
+      <c r="I219">
+        <v>1000</v>
+      </c>
+      <c r="J219" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="220" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>82</v>
+      </c>
+      <c r="B220" t="s">
+        <v>193</v>
+      </c>
+      <c r="C220" t="s">
+        <v>234</v>
+      </c>
+      <c r="I220">
+        <v>3000</v>
+      </c>
+      <c r="J220" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="221" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>241</v>
+      </c>
+      <c r="B221" t="s">
+        <v>242</v>
+      </c>
+      <c r="C221" t="s">
+        <v>234</v>
+      </c>
+      <c r="I221">
+        <v>400</v>
+      </c>
+      <c r="J221" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="222" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>99</v>
+      </c>
+      <c r="B222" t="s">
+        <v>210</v>
+      </c>
+      <c r="C222" t="s">
+        <v>234</v>
+      </c>
+      <c r="I222">
+        <v>100</v>
+      </c>
+      <c r="J222" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="223" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>100</v>
+      </c>
+      <c r="B223" t="s">
+        <v>211</v>
+      </c>
+      <c r="C223" t="s">
+        <v>234</v>
+      </c>
+      <c r="I223">
+        <v>100</v>
+      </c>
+      <c r="J223" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="224" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>101</v>
+      </c>
+      <c r="B224" t="s">
+        <v>212</v>
+      </c>
+      <c r="C224" t="s">
+        <v>234</v>
+      </c>
+      <c r="I224">
+        <v>100</v>
+      </c>
+      <c r="J224" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="225" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>251</v>
+      </c>
+      <c r="B225" t="s">
+        <v>252</v>
+      </c>
+      <c r="C225" t="s">
+        <v>234</v>
+      </c>
+      <c r="I225">
+        <v>50</v>
+      </c>
+      <c r="J225" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="226" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>91</v>
+      </c>
+      <c r="B226" t="s">
+        <v>202</v>
+      </c>
+      <c r="C226" t="s">
+        <v>234</v>
+      </c>
+      <c r="I226">
+        <v>3004</v>
+      </c>
+      <c r="J226" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="227" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>121</v>
+      </c>
+      <c r="B227" t="s">
+        <v>232</v>
+      </c>
+      <c r="C227" t="s">
+        <v>234</v>
+      </c>
+      <c r="I227">
+        <v>400</v>
+      </c>
+      <c r="J227" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="228" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
         <v>253</v>
       </c>
-      <c r="K207" s="8"/>
-    </row>
-    <row r="208" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A208" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B208" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C208" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I208" s="9">
+      <c r="C228" t="s">
+        <v>234</v>
+      </c>
+      <c r="I228">
+        <v>510</v>
+      </c>
+      <c r="J228" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="229" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>254</v>
+      </c>
+      <c r="C229" t="s">
+        <v>234</v>
+      </c>
+      <c r="I229">
+        <v>510</v>
+      </c>
+      <c r="J229" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="230" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>255</v>
+      </c>
+      <c r="C230" t="s">
+        <v>234</v>
+      </c>
+      <c r="I230">
         <v>500</v>
       </c>
-      <c r="J208" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K208" s="8"/>
-    </row>
-    <row r="209" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B209" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="C209" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I209" s="9">
+      <c r="J230" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="231" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>256</v>
+      </c>
+      <c r="C231" t="s">
+        <v>234</v>
+      </c>
+      <c r="I231">
+        <v>504</v>
+      </c>
+      <c r="J231" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="232" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>257</v>
+      </c>
+      <c r="C232" t="s">
+        <v>234</v>
+      </c>
+      <c r="I232">
+        <v>60</v>
+      </c>
+      <c r="J232" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="233" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>258</v>
+      </c>
+      <c r="C233" t="s">
+        <v>234</v>
+      </c>
+      <c r="I233">
         <v>1000</v>
       </c>
-      <c r="J209" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K209" s="8"/>
-    </row>
-    <row r="210" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B210" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="C210" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I210" s="9">
+      <c r="J233" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="234" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>259</v>
+      </c>
+      <c r="C234" t="s">
+        <v>234</v>
+      </c>
+      <c r="I234">
+        <v>100</v>
+      </c>
+      <c r="J234" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="235" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>260</v>
+      </c>
+      <c r="C235" t="s">
+        <v>234</v>
+      </c>
+      <c r="I235">
+        <v>100</v>
+      </c>
+      <c r="J235" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="236" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>261</v>
+      </c>
+      <c r="C236" t="s">
+        <v>234</v>
+      </c>
+      <c r="I236">
+        <v>100</v>
+      </c>
+      <c r="J236" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="237" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>262</v>
+      </c>
+      <c r="C237" t="s">
+        <v>234</v>
+      </c>
+      <c r="I237">
+        <v>100</v>
+      </c>
+      <c r="J237" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="238" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>263</v>
+      </c>
+      <c r="C238" t="s">
+        <v>234</v>
+      </c>
+      <c r="I238">
+        <v>100</v>
+      </c>
+      <c r="J238" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="239" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>264</v>
+      </c>
+      <c r="C239" t="s">
+        <v>234</v>
+      </c>
+      <c r="I239">
+        <v>50</v>
+      </c>
+      <c r="J239" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="240" spans="1:10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>315</v>
+      </c>
+      <c r="C240" t="s">
+        <v>234</v>
+      </c>
+      <c r="I240">
         <v>1000</v>
       </c>
-      <c r="J210" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K210" s="8"/>
-    </row>
-    <row r="211" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B211" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="C211" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I211" s="9">
-        <v>2010</v>
-      </c>
-      <c r="J211" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K211" s="8"/>
-    </row>
-    <row r="212" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B212" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C212" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I212" s="9">
-        <v>504</v>
-      </c>
-      <c r="J212" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K212" s="8"/>
-    </row>
-    <row r="213" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A213" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B213" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C213" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I213" s="9">
-        <v>501</v>
-      </c>
-      <c r="J213" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K213" s="8"/>
-    </row>
-    <row r="214" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B214" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C214" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I214" s="9">
-        <v>504</v>
-      </c>
-      <c r="J214" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K214" s="8"/>
-    </row>
-    <row r="215" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A215" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B215" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C215" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I215" s="9">
-        <v>1000</v>
-      </c>
-      <c r="J215" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K215" s="8"/>
-    </row>
-    <row r="216" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A216" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B216" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C216" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I216" s="9">
-        <v>480</v>
-      </c>
-      <c r="J216" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K216" s="8"/>
-    </row>
-    <row r="217" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A217" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B217" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C217" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I217" s="9">
-        <v>504</v>
-      </c>
-      <c r="J217" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K217" s="8"/>
-    </row>
-    <row r="218" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A218" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B218" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C218" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I218" s="9">
-        <v>500</v>
-      </c>
-      <c r="J218" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K218" s="8"/>
-    </row>
-    <row r="219" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A219" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B219" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C219" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I219" s="9">
-        <v>1000</v>
-      </c>
-      <c r="J219" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K219" s="8"/>
-    </row>
-    <row r="220" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A220" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B220" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C220" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I220" s="9">
-        <v>3000</v>
-      </c>
-      <c r="J220" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K220" s="8"/>
-    </row>
-    <row r="221" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A221" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="B221" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="C221" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I221" s="9">
-        <v>400</v>
-      </c>
-      <c r="J221" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K221" s="8"/>
-    </row>
-    <row r="222" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A222" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B222" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="C222" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I222" s="9">
-        <v>100</v>
-      </c>
-      <c r="J222" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K222" s="8"/>
-    </row>
-    <row r="223" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A223" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B223" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="C223" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I223" s="9">
-        <v>100</v>
-      </c>
-      <c r="J223" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K223" s="8"/>
-    </row>
-    <row r="224" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A224" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B224" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="C224" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I224" s="9">
-        <v>100</v>
-      </c>
-      <c r="J224" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K224" s="8"/>
-    </row>
-    <row r="225" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A225" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="B225" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="C225" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I225" s="9">
-        <v>50</v>
-      </c>
-      <c r="J225" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K225" s="8"/>
-    </row>
-    <row r="226" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A226" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B226" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C226" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I226" s="9">
-        <v>3004</v>
-      </c>
-      <c r="J226" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K226" s="8"/>
-    </row>
-    <row r="227" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A227" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B227" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="C227" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I227" s="9">
-        <v>400</v>
-      </c>
-      <c r="J227" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K227" s="8"/>
-    </row>
-    <row r="228" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A228" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="B228" s="3"/>
-      <c r="C228" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I228" s="9">
-        <v>510</v>
-      </c>
-      <c r="J228" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K228" s="8"/>
-    </row>
-    <row r="229" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A229" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="B229" s="3"/>
-      <c r="C229" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I229" s="9">
-        <v>510</v>
-      </c>
-      <c r="J229" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K229" s="8"/>
-    </row>
-    <row r="230" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A230" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="B230" s="3"/>
-      <c r="C230" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I230" s="9">
-        <v>500</v>
-      </c>
-      <c r="J230" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K230" s="8"/>
-    </row>
-    <row r="231" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A231" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="B231" s="3"/>
-      <c r="C231" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I231" s="9">
-        <v>504</v>
-      </c>
-      <c r="J231" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K231" s="8"/>
-    </row>
-    <row r="232" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A232" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="B232" s="3"/>
-      <c r="C232" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I232" s="9">
-        <v>60</v>
-      </c>
-      <c r="J232" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K232" s="8"/>
-    </row>
-    <row r="233" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A233" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="B233" s="3"/>
-      <c r="C233" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I233" s="9">
-        <v>1000</v>
-      </c>
-      <c r="J233" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K233" s="8"/>
-    </row>
-    <row r="234" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A234" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="B234" s="3"/>
-      <c r="C234" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I234" s="9">
-        <v>100</v>
-      </c>
-      <c r="J234" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K234" s="8"/>
-    </row>
-    <row r="235" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A235" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="B235" s="3"/>
-      <c r="C235" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I235" s="9">
-        <v>100</v>
-      </c>
-      <c r="J235" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K235" s="8"/>
-    </row>
-    <row r="236" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A236" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="B236" s="3"/>
-      <c r="C236" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I236" s="9">
-        <v>100</v>
-      </c>
-      <c r="J236" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K236" s="8"/>
-    </row>
-    <row r="237" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A237" s="10" t="s">
-        <v>263</v>
-      </c>
-      <c r="B237" s="3"/>
-      <c r="C237" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I237" s="9">
-        <v>100</v>
-      </c>
-      <c r="J237" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K237" s="8"/>
-    </row>
-    <row r="238" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A238" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="B238" s="3"/>
-      <c r="C238" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I238" s="9">
-        <v>100</v>
-      </c>
-      <c r="J238" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K238" s="8"/>
-    </row>
-    <row r="239" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A239" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="B239" s="3"/>
-      <c r="C239" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I239" s="9">
-        <v>50</v>
-      </c>
-      <c r="J239" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K239" s="8"/>
-    </row>
-    <row r="240" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A240" s="10" t="s">
+      <c r="J240" t="s">
         <v>317</v>
       </c>
-      <c r="B240" s="3"/>
-      <c r="C240" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="I240" s="9">
-        <v>1000</v>
-      </c>
-      <c r="J240" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="K240" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L240" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A2:A122">
+    <cfRule type="duplicateValues" dxfId="15" priority="2226"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A87">
+    <cfRule type="duplicateValues" dxfId="14" priority="2224"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A123:A124">
+    <cfRule type="duplicateValues" dxfId="13" priority="2217"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A125">
-    <cfRule type="duplicateValues" dxfId="17" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A182:A187">
+    <cfRule type="duplicateValues" dxfId="11" priority="2215"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A182:A193">
+    <cfRule type="duplicateValues" dxfId="10" priority="2216"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A195">
-    <cfRule type="duplicateValues" dxfId="16" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="13" priority="1919"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1919"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="12" priority="2130"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="2131" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2130"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2131" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="10" priority="1917"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="1918" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1917"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1918" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="8" priority="1915"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="1916" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A207:A220">
-    <cfRule type="duplicateValues" dxfId="6" priority="2195"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A196:A199">
-    <cfRule type="duplicateValues" dxfId="5" priority="2196"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A182:A187">
-    <cfRule type="duplicateValues" dxfId="4" priority="2215"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A182:A193">
-    <cfRule type="duplicateValues" dxfId="3" priority="2216"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A123:A124">
-    <cfRule type="duplicateValues" dxfId="2" priority="2217"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A87">
-    <cfRule type="duplicateValues" dxfId="1" priority="2224"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A122">
-    <cfRule type="duplicateValues" dxfId="0" priority="2226"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1915"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1916" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>